<commit_message>
BID RC-V: troca Observações por um campo para cada informação
Novas colunas: seguradora atual, modalidade, custo por viagem, base de
viagens, parcelamento, IOF, custos de defesa, outras coberturas,
veículo vazio, cláusula de revisão, cotação do DES, início de
vigência, validade da proposta e fonte da informação.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FuMPiQvjswbB9c7eCTcVzg
</commit_message>
<xml_diff>
--- a/BID-preenchido/BID RC-V.xlsx
+++ b/BID-preenchido/BID RC-V.xlsx
@@ -305,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -447,6 +447,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -800,7 +803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63DC7E7-4034-4135-A538-7E63B5C055B5}">
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -812,16 +815,28 @@
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="40" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="14" width="26" customWidth="1"/>
-    <col min="15" max="15" width="60" customWidth="1"/>
-    <col min="16" max="16" width="18.140625" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="30" customWidth="1"/>
+    <col min="23" max="23" width="26" customWidth="1"/>
+    <col min="24" max="24" width="28" customWidth="1"/>
+    <col min="25" max="25" width="18" customWidth="1"/>
+    <col min="26" max="26" width="19" customWidth="1"/>
+    <col min="27" max="27" width="22" customWidth="1"/>
+    <col min="28" max="28" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
         <v>5</v>
       </c>
@@ -840,8 +855,20 @@
       <c r="N1" s="35"/>
       <c r="O1" s="35"/>
       <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="35"/>
+      <c r="Y1" s="35"/>
+      <c r="Z1" s="35"/>
+      <c r="AA1" s="35"/>
+      <c r="AB1" s="35"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="32" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
@@ -884,14 +911,78 @@
       <c r="N2" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="O2" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OBSERVAÇÕES</t>
-        </is>
-      </c>
-      <c r="P2" s="17"/>
+      <c r="O2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEGURADORA ATUAL</t>
+        </is>
+      </c>
+      <c r="P2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MODALIDADE</t>
+        </is>
+      </c>
+      <c r="Q2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CUSTO POR VIAGEM</t>
+        </is>
+      </c>
+      <c r="R2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BASE DE VIAGENS</t>
+        </is>
+      </c>
+      <c r="S2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARCELAMENTO</t>
+        </is>
+      </c>
+      <c r="T2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IOF</t>
+        </is>
+      </c>
+      <c r="U2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CUSTOS DE DEFESA</t>
+        </is>
+      </c>
+      <c r="V2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUTRAS COBERTURAS ADICIONAIS</t>
+        </is>
+      </c>
+      <c r="W2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VEÍCULO VAZIO</t>
+        </is>
+      </c>
+      <c r="X2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLÁUSULA DE REVISÃO</t>
+        </is>
+      </c>
+      <c r="Y2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COTAÇÃO DO DES</t>
+        </is>
+      </c>
+      <c r="Z2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INÍCIO DE VIGÊNCIA</t>
+        </is>
+      </c>
+      <c r="AA2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDADE DA PROPOSTA</t>
+        </is>
+      </c>
+      <c r="AB2" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FONTE DA INFORMAÇÃO</t>
+        </is>
+      </c>
     </row>
-    <row r="3" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -931,8 +1022,7 @@
       </c>
       <c r="J3" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 meses
-(ajustável)</t>
+          <t xml:space="preserve">12 meses</t>
         </is>
       </c>
       <c r="K3" s="36" t="inlineStr">
@@ -943,8 +1033,7 @@
       </c>
       <c r="L3" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">R$ 266.112,00
-(25.344 viagens × R$ 10,50)</t>
+          <t xml:space="preserve">R$ 266.112,00</t>
         </is>
       </c>
       <c r="M3" s="36" t="inlineStr">
@@ -959,11 +1048,78 @@
       </c>
       <c r="O3" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposta Gallagher (quadro resumo). Prêmios líquidos, + IOF 7,38%. Até 10x sem juros.</t>
+          <t xml:space="preserve">Não
+(detentora do RCF-V)</t>
+        </is>
+      </c>
+      <c r="P3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável</t>
+        </is>
+      </c>
+      <c r="Q3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$ 10,50</t>
+        </is>
+      </c>
+      <c r="R3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.344/ano
+(2.112/mês)</t>
+        </is>
+      </c>
+      <c r="S3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Até 10x sem juros</t>
+        </is>
+      </c>
+      <c r="T3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="V3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="W3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="X3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="Z3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AA3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AB3" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quadro resumo da Gallagher</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
       <c r="C4" s="4" t="s">
@@ -997,8 +1153,7 @@
       </c>
       <c r="J4" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 ou 24 meses
-(ajustável)</t>
+          <t xml:space="preserve">12 ou 24 meses</t>
         </is>
       </c>
       <c r="K4" s="37" t="inlineStr">
@@ -1009,8 +1164,9 @@
       </c>
       <c r="L4" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">12m: R$ 88.704,00 (R$ 3,50/viagem)
-24m: R$ 152.064,00 total = R$ 76.032,00/ano (R$ 3,00/viagem)</t>
+          <t xml:space="preserve">12m: R$ 88.704,00
+24m: R$ 152.064,00
+(R$ 76.032,00/ano)</t>
         </is>
       </c>
       <c r="M4" s="37" t="inlineStr">
@@ -1025,11 +1181,80 @@
       </c>
       <c r="O4" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proposta Gallagher (quadro resumo). Prêmios líquidos, + IOF 7,38%. 12m até 10x; 24m até 20x sem juros.</t>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="P4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável</t>
+        </is>
+      </c>
+      <c r="Q4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: R$ 3,50
+24m: R$ 3,00</t>
+        </is>
+      </c>
+      <c r="R4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.344/ano
+(2.112/mês)</t>
+        </is>
+      </c>
+      <c r="S4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: até 10x
+24m: até 20x
+(sem juros)</t>
+        </is>
+      </c>
+      <c r="T4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="V4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="W4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="X4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aplicável só a vigência &gt; 12 meses</t>
+        </is>
+      </c>
+      <c r="Y4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="Z4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AA4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AB4" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quadro resumo da Gallagher</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
       <c r="C5" s="4" t="s">
@@ -1059,13 +1284,12 @@
       <c r="I5" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">R$ 30.000,00
-(franquia isenta)</t>
+(isento de franquia)</t>
         </is>
       </c>
       <c r="J5" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 ou 24 meses
-(ajustável)</t>
+          <t xml:space="preserve">12 ou 24 meses</t>
         </is>
       </c>
       <c r="K5" s="37" t="inlineStr">
@@ -1076,8 +1300,9 @@
       </c>
       <c r="L5" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">12m: R$ 63.360,00 (R$ 2,50/viagem)
-24m: R$ 108.979,20 total = R$ 54.489,60/ano (R$ 2,15/viagem)</t>
+          <t xml:space="preserve">12m: R$ 63.360,00
+24m: R$ 108.979,20
+(R$ 54.489,60/ano)</t>
         </is>
       </c>
       <c r="M5" s="37" t="inlineStr">
@@ -1093,11 +1318,82 @@
       </c>
       <c r="O5" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Única proposta na íntegra da Gallagher. Prêmios líquidos, + IOF 7,38%. 12m até 10x; 24m até 20x sem juros. Cláusula de revisão p/ vigência &gt; 12m; reanálise bimestral se S/P &gt; 50%. Validade 30 dias (carta de 08/10/2026).</t>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="P5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável</t>
+        </is>
+      </c>
+      <c r="Q5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: R$ 2,50
+24m: R$ 2,15</t>
+        </is>
+      </c>
+      <c r="R5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.344/ano no quadro resumo
+(a proposta AXA cita 37.131 embarques/ano)</t>
+        </is>
+      </c>
+      <c r="S5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: até 10x
+24m: até 20x
+(sem juros)</t>
+        </is>
+      </c>
+      <c r="T5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não contempla</t>
+        </is>
+      </c>
+      <c r="V5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coberto da ordem de coleta até a coleta</t>
+        </is>
+      </c>
+      <c r="X5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vigência &gt; 12m: revisão
+Reanálise bimestral se S/P &gt; 50%</t>
+        </is>
+      </c>
+      <c r="Y5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convertido na data do embarque</t>
+        </is>
+      </c>
+      <c r="Z5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AA5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 dias
+(carta de 08/10/2026)</t>
+        </is>
+      </c>
+      <c r="AB5" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposta AXA na íntegra (Gallagher)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="30" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="5" t="s">
@@ -1152,11 +1448,76 @@
       </c>
       <c r="O6" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem cotação desta seguradora na proposta da Gallagher</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="P6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Q6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="S6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="T6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="U6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="V6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="X6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Z6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AA6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AB6" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sem cotação na proposta da Gallagher</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1197,8 +1558,7 @@
       </c>
       <c r="J7" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 ou 24 meses
-(averbável)</t>
+          <t xml:space="preserve">12 ou 24 meses</t>
         </is>
       </c>
       <c r="K7" s="36" t="inlineStr">
@@ -1209,15 +1569,14 @@
       </c>
       <c r="L7" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">12m: R$ 5,50/viagem
-24m: R$ 5,00/viagem
-(est. 25.344 viagens: R$ 139.392,00/ano 12m; R$ 126.720,00/ano 24m)</t>
+          <t xml:space="preserve">Estimado:
+12m: R$ 139.392,00/ano
+24m: R$ 126.720,00/ano</t>
         </is>
       </c>
       <c r="M7" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">R$ 350,00/mês
-+ IOF</t>
+          <t xml:space="preserve">R$ 350,00/mês</t>
         </is>
       </c>
       <c r="N7" s="36" t="inlineStr">
@@ -1228,11 +1587,78 @@
       </c>
       <c r="O7" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detentora atual. DES a R$ 8,00. Sem custos de defesa. Exclui veículo vazio / retorno após entrega. Estimativa anual calculada com as 25.344 viagens usadas pelas demais corretoras.</t>
+          <t xml:space="preserve">Sim (RC-V)</t>
+        </is>
+      </c>
+      <c r="P7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Averbável</t>
+        </is>
+      </c>
+      <c r="Q7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: R$ 5,50
+24m: R$ 5,00</t>
+        </is>
+      </c>
+      <c r="R7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado
+(estimativa com 25.344/ano)</t>
+        </is>
+      </c>
+      <c r="S7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fatura mensal</t>
+        </is>
+      </c>
+      <c r="T7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não possui</t>
+        </is>
+      </c>
+      <c r="V7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excluído (inclusive retorno após entrega)</t>
+        </is>
+      </c>
+      <c r="X7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="Y7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$ 8,00</t>
+        </is>
+      </c>
+      <c r="Z7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30/10/2026</t>
+        </is>
+      </c>
+      <c r="AA7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Até 25/10/2026</t>
+        </is>
+      </c>
+      <c r="AB7" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposta de renovação AON</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="30" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="10"/>
       <c r="C8" s="12" t="s">
@@ -1289,11 +1715,76 @@
       </c>
       <c r="O8" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem cotação desta seguradora na proposta da AON</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="P8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Q8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="S8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="T8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="U8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="V8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="X8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Z8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AA8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AB8" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sem cotação na proposta da AON</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="11"/>
       <c r="C9" s="14" t="s">
@@ -1325,8 +1816,7 @@
       </c>
       <c r="J9" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 ou 24 meses
-(averbável; 24m via LTA)</t>
+          <t xml:space="preserve">12 ou 24 meses</t>
         </is>
       </c>
       <c r="K9" s="38" t="inlineStr">
@@ -1337,15 +1827,14 @@
       </c>
       <c r="L9" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">12m: R$ 4,00/viagem
-24m: R$ 3,50/viagem
-(est. 25.344 viagens: R$ 101.376,00/ano 12m; R$ 88.704,00/ano 24m)</t>
+          <t xml:space="preserve">Estimado:
+12m: R$ 101.376,00/ano
+24m: R$ 88.704,00/ano</t>
         </is>
       </c>
       <c r="M9" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">R$ 350,00/mês
-+ IOF</t>
+          <t xml:space="preserve">R$ 350,00/mês</t>
         </is>
       </c>
       <c r="N9" s="38" t="inlineStr">
@@ -1355,11 +1844,78 @@
       </c>
       <c r="O9" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linha "A | G" = AIG Seguros. DES a R$ 8,00. Custos de defesa R$ 5.000,00/evento. LTA 24m: condições revistas se sinistralidade &gt; 60% no 1º ano. Início previsto 30/10/2026.</t>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="P9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Averbável</t>
+        </is>
+      </c>
+      <c r="Q9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12m: R$ 4,00
+24m: R$ 3,50</t>
+        </is>
+      </c>
+      <c r="R9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado
+(estimativa com 25.344/ano)</t>
+        </is>
+      </c>
+      <c r="S9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fatura mensal</t>
+        </is>
+      </c>
+      <c r="T9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$ 5.000,00/evento</t>
+        </is>
+      </c>
+      <c r="V9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coberto só na coleta anterior à viagem</t>
+        </is>
+      </c>
+      <c r="X9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24m (LTA): revisão se sinistralidade &gt; 60% no 1º ano</t>
+        </is>
+      </c>
+      <c r="Y9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$ 8,00</t>
+        </is>
+      </c>
+      <c r="Z9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30/10/2026</t>
+        </is>
+      </c>
+      <c r="AA9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Até 25/10/2026</t>
+        </is>
+      </c>
+      <c r="AB9" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposta de renovação AON</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" ht="80" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>20</v>
       </c>
@@ -1407,8 +1963,8 @@
       </c>
       <c r="L10" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ajustável: R$ 76.032,00 (25.344 viagens × R$ 3,00)
-Averbável: R$ 4,00/viagem</t>
+          <t xml:space="preserve">Ajustável: R$ 76.032,00
+Averbável: conforme viagens</t>
         </is>
       </c>
       <c r="M10" s="36" t="inlineStr">
@@ -1425,11 +1981,78 @@
       </c>
       <c r="O10" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Via Albatroz MGA. Cobre frota própria inclusive retorno vazio. Sem custo adicional: AP motorista R$ 10.000 e custas de defesa R$ 10.000. Prêmios líquidos, + IOF 7,38%. Até 10x. Ajustável sem devolução em cancelamento.</t>
+          <t xml:space="preserve">Não</t>
+        </is>
+      </c>
+      <c r="P10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável ou averbável</t>
+        </is>
+      </c>
+      <c r="Q10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável: R$ 3,00
+Averbável: R$ 4,00</t>
+        </is>
+      </c>
+      <c r="R10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.344/ano</t>
+        </is>
+      </c>
+      <c r="S10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Até 10x</t>
+        </is>
+      </c>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7,38%</t>
+        </is>
+      </c>
+      <c r="U10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R$ 10.000,00
+(sem custo)</t>
+        </is>
+      </c>
+      <c r="V10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AP motorista (morte / funeral): R$ 10.000,00 (sem custo)</t>
+        </is>
+      </c>
+      <c r="W10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coberto até a coleta; frota própria também no retorno vazio</t>
+        </is>
+      </c>
+      <c r="X10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajustável: acerto final pelas viagens reais; sem devolução se cancelar</t>
+        </is>
+      </c>
+      <c r="Y10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="Z10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Não informado</t>
+        </is>
+      </c>
+      <c r="AA10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 dias</t>
+        </is>
+      </c>
+      <c r="AB10" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duas propostas Alper (Albatroz MGA)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" ht="30" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="19"/>
       <c r="B11" s="21"/>
       <c r="C11" s="12" t="s">
@@ -1484,11 +2107,76 @@
       </c>
       <c r="O11" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sem cotação desta seguradora na proposta da Alper</t>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="P11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Q11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="S11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="T11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="U11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="V11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="X11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Z11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AA11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AB11" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sem cotação na proposta da Alper</t>
         </is>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>22</v>
       </c>
@@ -1533,11 +2221,76 @@
       </c>
       <c r="O12" s="36" t="inlineStr">
         <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="P12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Q12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="S12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="U12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="V12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="X12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Z12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AA12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AB12" s="36" t="inlineStr">
+        <is>
           <t xml:space="preserve">Não apresentou proposta</t>
         </is>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19"/>
       <c r="B13" s="25"/>
       <c r="C13" s="14" t="s">
@@ -1559,8 +2312,73 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="P13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Z13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB13" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
-    <row r="14" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>17</v>
       </c>
@@ -1605,11 +2423,76 @@
       </c>
       <c r="O14" s="36" t="inlineStr">
         <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="P14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Q14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="S14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="T14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="U14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="V14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="W14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="X14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Y14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="Z14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AA14" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="AB14" s="36" t="inlineStr">
+        <is>
           <t xml:space="preserve">Não apresentou proposta</t>
         </is>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19"/>
       <c r="B15" s="8"/>
       <c r="C15" s="14" t="s">
@@ -1631,9 +2514,74 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="P15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Q15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="U15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="V15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="W15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="X15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Y15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="Z15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AB15" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="62">
     <mergeCell ref="M12:M13"/>
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="G12:G13"/>
@@ -1659,7 +2607,7 @@
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="E12:E13"/>
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:AB1"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="A7:A9"/>
@@ -1670,6 +2618,32 @@
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="O12:O13"/>
     <mergeCell ref="O14:O15"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q12:Q13"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="R12:R13"/>
+    <mergeCell ref="R14:R15"/>
+    <mergeCell ref="S12:S13"/>
+    <mergeCell ref="S14:S15"/>
+    <mergeCell ref="T12:T13"/>
+    <mergeCell ref="T14:T15"/>
+    <mergeCell ref="U12:U13"/>
+    <mergeCell ref="U14:U15"/>
+    <mergeCell ref="V12:V13"/>
+    <mergeCell ref="V14:V15"/>
+    <mergeCell ref="W12:W13"/>
+    <mergeCell ref="W14:W15"/>
+    <mergeCell ref="X12:X13"/>
+    <mergeCell ref="X14:X15"/>
+    <mergeCell ref="Y12:Y13"/>
+    <mergeCell ref="Y14:Y15"/>
+    <mergeCell ref="Z12:Z13"/>
+    <mergeCell ref="Z14:Z15"/>
+    <mergeCell ref="AA12:AA13"/>
+    <mergeCell ref="AA14:AA15"/>
+    <mergeCell ref="AB12:AB13"/>
+    <mergeCell ref="AB14:AB15"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>